<commit_message>
Convert flashcards to multiple choice
Cards are now single-answer multiple choice (topic, question, options,
correctIndex) instead of free-text Q&A with self-grading. Study
sessions grade automatically on selection, highlighting the correct
answer and the user's choice if wrong. Updates the manage-card form,
JSON import/export shape, spreadsheet template and parser (Option
A-D + Correct Option columns), starter deck, and README accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QdEjUnYNPuH8SCWDRGrjY8
</commit_message>
<xml_diff>
--- a/data/flashcard-template.xlsx
+++ b/data/flashcard-template.xlsx
@@ -450,12 +450,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -471,7 +475,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Option C</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Option D</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct Option</t>
         </is>
       </c>
     </row>
@@ -483,12 +507,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>What is the difference between a Profile and a Permission Set?</t>
+          <t>Which single component must every Salesforce user be assigned exactly one of, to set their baseline object, field, and app permissions?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A Profile is a single, required baseline of permissions assigned to a user; a Permission Set grants additional permissions on top of it, and a user can have multiple.</t>
+          <t>Permission Set</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Permission Set Group</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Public Group</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -500,12 +544,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>What is the recommended tool for record-triggered automation today?</t>
+          <t>Which Salesforce automation tool is now recommended for record-triggered logic, replacing Workflow Rules and Process Builder?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Flow (specifically Record-Triggered Flow), which has replaced Workflow Rules and Process Builder.</t>
+          <t>Approval Processes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Apex Triggers</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Validation Rules</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -517,12 +581,32 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>What tool should you use to import or update more than 50,000 records?</t>
+          <t>Which tool should an admin use to insert or update more than 50,000 records at once?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Data Loader, since it uses the Bulk API and has no 50,000-record cap like the Data Import Wizard.</t>
+          <t>Data Import Wizard</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Report Export</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Change Sets</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -530,101 +614,181 @@
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
       <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -637,10 +801,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -656,7 +820,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. On the "Flashcards" tab, keep the header row (Topic, Question, Answer) as-is.</t>
+          <t>1. On the "Flashcards" tab, keep the header row as-is: Topic, Question, Option A, Option B, Option C, Option D, Correct Option.</t>
         </is>
       </c>
     </row>
@@ -670,43 +834,57 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>3. Add one flashcard per row: a short Topic label, the Question, and the Answer.</t>
+          <t>3. Add one multiple-choice question per row: a short Topic label, the Question, four answer Options, and which one is correct.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>4. Save the file as .xlsx or .csv.</t>
+          <t>4. "Correct Option" must be the letter A, B, C, or D — matching the column of the right answer.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>5. In the app's "Manage Cards" tab, use "Upload Spreadsheet" and select this file.</t>
+          <t>5. Save the file as .xlsx or .csv.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>6. In the app's "Manage Cards" tab, use "Upload a Spreadsheet" and select this file.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Tips:</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
+          <t>Tips:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>- Only one option should be correct per question — this app scores single-answer multiple choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>- Leave a row completely blank to skip it — blank rows are ignored on import.</t>
         </is>

</xml_diff>

<commit_message>
Support 4-8 answer options per question
Real exam questions don't always have exactly 4 choices, so cards now
support 4-8 options instead of a fixed 4. The Manage Cards form starts
with 4 option fields and lets you add up to 8 (with per-row remove
buttons); the spreadsheet template gains Option E-H columns (left
blank when unused); JSON import/export and the study-session renderer
already worked off the options array length, so they scale naturally.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QdEjUnYNPuH8SCWDRGrjY8
</commit_message>
<xml_diff>
--- a/data/flashcard-template.xlsx
+++ b/data/flashcard-template.xlsx
@@ -450,16 +450,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -495,6 +498,26 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Option E</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Option F</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Option G</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Option H</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Correct Option</t>
         </is>
       </c>
@@ -530,7 +553,11 @@
           <t>Public Group</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -539,74 +566,106 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Data Management</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Which Salesforce automation tool is now recommended for record-triggered logic, replacing Workflow Rules and Process Builder?</t>
+          <t>Which tool should an admin use to insert or update more than 50,000 records at once?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Approval Processes</t>
+          <t>Data Import Wizard</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Apex Triggers</t>
+          <t>Data Loader</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Report Export</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Validation Rules</t>
+          <t>Change Sets</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Path Assistant</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate Rules</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Data Management</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Which tool should an admin use to insert or update more than 50,000 records at once?</t>
+          <t>Which Salesforce automation tool is now recommended for record-triggered logic, replacing Workflow Rules and Process Builder?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Data Import Wizard</t>
+          <t>Approval Processes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Data Loader</t>
+          <t>Apex Triggers</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Report Export</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Change Sets</t>
+          <t>Validation Rules</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Escalation Rules</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Assignment Rules</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Macros</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Quick Actions</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
@@ -618,6 +677,10 @@
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -627,6 +690,10 @@
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -636,6 +703,10 @@
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -645,6 +716,10 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -654,6 +729,10 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -663,6 +742,10 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -672,6 +755,10 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -681,6 +768,10 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -690,6 +781,10 @@
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -699,6 +794,10 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -708,6 +807,10 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -717,6 +820,10 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -726,6 +833,10 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -735,6 +846,10 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -744,6 +859,10 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -753,6 +872,10 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -762,6 +885,10 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -771,6 +898,10 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -780,6 +911,10 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -789,6 +924,10 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -801,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -820,7 +959,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. On the "Flashcards" tab, keep the header row as-is: Topic, Question, Option A, Option B, Option C, Option D, Correct Option.</t>
+          <t>1. On the "Flashcards" tab, keep the header row as-is: Topic, Question, Option A-H, Correct Option.</t>
         </is>
       </c>
     </row>
@@ -834,57 +973,64 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>3. Add one multiple-choice question per row: a short Topic label, the Question, four answer Options, and which one is correct.</t>
+          <t>3. Add one multiple-choice question per row: a short Topic label, the Question, and its answer Options.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>4. "Correct Option" must be the letter A, B, C, or D — matching the column of the right answer.</t>
+          <t>4. Each question can have anywhere from 4 to 8 options — just fill in Option A through however many you need (D, F, or H, for example) and leave the rest blank.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>5. Save the file as .xlsx or .csv.</t>
+          <t>5. "Correct Option" must be the letter (A-H) matching the column of the right answer.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6. In the app's "Manage Cards" tab, use "Upload a Spreadsheet" and select this file.</t>
+          <t>6. Save the file as .xlsx or .csv.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>7. In the app's "Manage Cards" tab, use "Upload a Spreadsheet" and select this file.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Tips:</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
+          <t>Tips:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>- Only one option should be correct per question — this app scores single-answer multiple choice.</t>
+          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>- Only one option should be correct per question — this app scores single-answer multiple choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>- Leave a row completely blank to skip it — blank rows are ignored on import.</t>
         </is>

</xml_diff>

<commit_message>
Support multi-answer "choose N" questions
Cards can now require selecting more than one correct option, matching
real exam questions like "Choose 2" or "Choose 3". The schema moves
from a single correctIndex to a correctIndexes array; single-answer
cards just have one entry and keep the existing instant-grade-on-click
flow. Multi-answer cards render as toggleable options with a "Select N
answers" hint and a Submit button, graded all-or-nothing (must pick
exactly the right set).

Updates the manage-card form (checkboxes instead of radios), JSON
import/export, the spreadsheet template and parser (Correct Option
accepts comma-separated letters), starter deck, and README.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QdEjUnYNPuH8SCWDRGrjY8
</commit_message>
<xml_diff>
--- a/data/flashcard-template.xlsx
+++ b/data/flashcard-template.xlsx
@@ -462,7 +462,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -620,52 +620,52 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Which Salesforce automation tool is now recommended for record-triggered logic, replacing Workflow Rules and Process Builder?</t>
+          <t>Which three of these are valid Flow trigger types? (Choose 3)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Approval Processes</t>
+          <t>Record-Triggered</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Apex Triggers</t>
+          <t>Schedule-Triggered</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Platform Event-Triggered</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Validation Rules</t>
+          <t>Report-Triggered</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>Macros</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Quick Actions</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Assignment Rules</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Escalation Rules</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Assignment Rules</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Macros</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Quick Actions</t>
-        </is>
-      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A, B, C</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -987,50 +987,64 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>5. "Correct Option" must be the letter (A-H) matching the column of the right answer.</t>
+          <t>5. "Correct Option" holds the letter(s) (A-H) of the right answer(s):</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6. Save the file as .xlsx or .csv.</t>
+          <t xml:space="preserve">   - Single-answer question: one letter, e.g. "C".</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>7. In the app's "Manage Cards" tab, use "Upload a Spreadsheet" and select this file.</t>
+          <t xml:space="preserve">   - "Choose N" question with multiple correct answers: every correct letter separated by commas, e.g. "A, C" or "B, D, E". The app then requires picking exactly that set to count it correct.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>6. Save the file as .xlsx or .csv.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Tips:</t>
+          <t>7. In the app's "Manage Cards" tab, use "Upload a Spreadsheet" and select this file.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>- Only one option should be correct per question — this app scores single-answer multiple choice.</t>
+          <t>Tips:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>- Reuse the same Topic spelling across rows (e.g. always "Security &amp; Access") so cards group together for topic mastery tracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>- For a "choose N" question, it helps to say so in the Question text itself (e.g. "...(Choose 2)") since the app will also show a "Select N answers" hint during study.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>- Leave a row completely blank to skip it — blank rows are ignored on import.</t>
         </is>

</xml_diff>